<commit_message>
Add product-card block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 17
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-eds-site.report.xlsx
+++ b/tools/importer/reports/import-eds-site.report.xlsx
@@ -70,7 +70,7 @@
     <t>en/accounts</t>
   </si>
   <si>
-    <t>2026-10-23T13:39:25.835Z</t>
+    <t>2026-10-23T18:26:20.565Z</t>
   </si>
   <si>
     <t>Accounts</t>
@@ -133,7 +133,7 @@
     <t>en/credit-cards</t>
   </si>
   <si>
-    <t>2026-10-23T13:37:55.625Z</t>
+    <t>2026-10-23T18:26:29.091Z</t>
   </si>
   <si>
     <t>Credit Cards</t>
@@ -202,7 +202,7 @@
     <t>en/insurance</t>
   </si>
   <si>
-    <t>2026-10-23T13:38:09.960Z</t>
+    <t>2026-10-23T18:26:55.481Z</t>
   </si>
   <si>
     <t>Insurance</t>
@@ -220,7 +220,7 @@
     <t>en/loans</t>
   </si>
   <si>
-    <t>2026-10-23T13:39:17.782Z</t>
+    <t>2026-10-23T18:27:08.053Z</t>
   </si>
   <si>
     <t>Loans</t>
@@ -361,7 +361,7 @@
     <t>en/credit-cards/credit-card-basic</t>
   </si>
   <si>
-    <t>2026-10-23T13:37:07.683Z</t>
+    <t>2026-10-23T18:26:34.114Z</t>
   </si>
   <si>
     <t>Credit Card Basic</t>
@@ -376,7 +376,7 @@
     <t>en/credit-cards/credit-card-gold</t>
   </si>
   <si>
-    <t>2026-10-23T13:37:42.193Z</t>
+    <t>2026-10-23T18:26:40.165Z</t>
   </si>
   <si>
     <t>Credit Card Gold</t>
@@ -391,7 +391,7 @@
     <t>en/credit-cards/credit-card-premium</t>
   </si>
   <si>
-    <t>2026-10-23T13:37:25.783Z</t>
+    <t>2026-10-23T18:26:44.979Z</t>
   </si>
   <si>
     <t>Credit Card Premium</t>
@@ -505,7 +505,7 @@
     <t>en/loans/car-loan</t>
   </si>
   <si>
-    <t>2026-10-23T13:38:41.633Z</t>
+    <t>2026-10-23T18:27:13.938Z</t>
   </si>
   <si>
     <t>Car Loan</t>
@@ -535,7 +535,7 @@
     <t>en/loans/home-loan</t>
   </si>
   <si>
-    <t>2026-10-23T13:38:02.287Z</t>
+    <t>2026-10-23T18:27:20.620Z</t>
   </si>
   <si>
     <t>Home Loan</t>
@@ -550,7 +550,7 @@
     <t>en/loans/personal-loan</t>
   </si>
   <si>
-    <t>2026-10-23T13:39:56.928Z</t>
+    <t>2026-10-23T18:27:26.295Z</t>
   </si>
   <si>
     <t>Personal Loan</t>
@@ -565,7 +565,7 @@
     <t>en/loans/student-loan</t>
   </si>
   <si>
-    <t>2026-10-23T13:39:01.952Z</t>
+    <t>2026-10-23T18:27:31.336Z</t>
   </si>
   <si>
     <t>Student Loan</t>

</xml_diff>